<commit_message>
Add default registry lab federation demos
</commit_message>
<xml_diff>
--- a/data/agriculture/agri-program-registry.xlsx
+++ b/data/agriculture/agri-program-registry.xlsx
@@ -794,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -810,6 +810,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -870,10 +871,15 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>valid_from</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>issued_on</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>expires_on</t>
         </is>
@@ -937,6 +943,9 @@
         <v>46113</v>
       </c>
       <c r="M2" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="N2" s="1" t="n">
         <v>46203</v>
       </c>
     </row>
@@ -998,6 +1007,9 @@
         <v>46114</v>
       </c>
       <c r="M3" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="N3" s="1" t="n">
         <v>46203</v>
       </c>
     </row>
@@ -1059,6 +1071,9 @@
         <v>46113</v>
       </c>
       <c r="M4" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="N4" s="1" t="n">
         <v>46203</v>
       </c>
     </row>
@@ -1120,6 +1135,9 @@
         <v>46115</v>
       </c>
       <c r="M5" s="1" t="n">
+        <v>46115</v>
+      </c>
+      <c r="N5" s="1" t="n">
         <v>46203</v>
       </c>
     </row>
@@ -1181,6 +1199,9 @@
         <v>46116</v>
       </c>
       <c r="M6" s="1" t="n">
+        <v>46116</v>
+      </c>
+      <c r="N6" s="1" t="n">
         <v>46203</v>
       </c>
     </row>

</xml_diff>